<commit_message>
Actualizacion final añadiendo usuario a los VL
</commit_message>
<xml_diff>
--- a/utiles/Tests caja negra.xlsx
+++ b/utiles/Tests caja negra.xlsx
@@ -4,21 +4,21 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4507"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="300" windowWidth="14880" windowHeight="7815"/>
+    <workbookView xWindow="360" yWindow="300" windowWidth="14880" windowHeight="7815" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="CE Reducido" sheetId="1" r:id="rId1"/>
     <sheet name="CE" sheetId="5" r:id="rId2"/>
     <sheet name="Pairwise" sheetId="3" r:id="rId3"/>
     <sheet name="VL Reducido" sheetId="6" r:id="rId4"/>
-    <sheet name="VL" sheetId="7" r:id="rId5"/>
+    <sheet name="VL Pairwise" sheetId="7" r:id="rId5"/>
   </sheets>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="155">
   <si>
     <t>Entrada</t>
   </si>
@@ -435,6 +435,54 @@
   </si>
   <si>
     <t>TC31</t>
+  </si>
+  <si>
+    <t>VL09</t>
+  </si>
+  <si>
+    <t>VL10</t>
+  </si>
+  <si>
+    <t>VL11</t>
+  </si>
+  <si>
+    <t>VL12</t>
+  </si>
+  <si>
+    <t>VL13</t>
+  </si>
+  <si>
+    <t>VL14</t>
+  </si>
+  <si>
+    <t>Usuario_VL</t>
+  </si>
+  <si>
+    <t>Contrasena</t>
+  </si>
+  <si>
+    <t>TC32</t>
+  </si>
+  <si>
+    <t>TC33</t>
+  </si>
+  <si>
+    <t>TC34</t>
+  </si>
+  <si>
+    <t>TC35</t>
+  </si>
+  <si>
+    <t>TC36</t>
+  </si>
+  <si>
+    <t>TC37</t>
+  </si>
+  <si>
+    <t>abcd</t>
+  </si>
+  <si>
+    <t>abcde</t>
   </si>
 </sst>
 </file>
@@ -625,7 +673,7 @@
       <protection locked="0"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -665,9 +713,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -694,6 +740,10 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1012,7 +1062,7 @@
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="33" t="s">
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1024,7 +1074,7 @@
       <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="35"/>
+      <c r="A3" s="33"/>
       <c r="B3" s="2" t="s">
         <v>34</v>
       </c>
@@ -1034,7 +1084,7 @@
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="35"/>
+      <c r="A4" s="33"/>
       <c r="B4" s="2" t="s">
         <v>38</v>
       </c>
@@ -1044,7 +1094,7 @@
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" s="35"/>
+      <c r="A5" s="33"/>
       <c r="B5" s="2" t="s">
         <v>40</v>
       </c>
@@ -1060,7 +1110,7 @@
       <c r="D6" s="24"/>
     </row>
     <row r="7" spans="1:4">
-      <c r="A7" s="34" t="s">
+      <c r="A7" s="32" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -1072,7 +1122,7 @@
       </c>
     </row>
     <row r="8" spans="1:4">
-      <c r="A8" s="34"/>
+      <c r="A8" s="32"/>
       <c r="B8" s="3" t="s">
         <v>46</v>
       </c>
@@ -1082,7 +1132,7 @@
       <c r="D8" s="3"/>
     </row>
     <row r="9" spans="1:4">
-      <c r="A9" s="34"/>
+      <c r="A9" s="32"/>
       <c r="B9" s="2" t="s">
         <v>48</v>
       </c>
@@ -1092,7 +1142,7 @@
       </c>
     </row>
     <row r="10" spans="1:4">
-      <c r="A10" s="34"/>
+      <c r="A10" s="32"/>
       <c r="B10" s="2" t="s">
         <v>50</v>
       </c>
@@ -1102,7 +1152,7 @@
       </c>
     </row>
     <row r="11" spans="1:4">
-      <c r="A11" s="34"/>
+      <c r="A11" s="32"/>
       <c r="B11" s="2" t="s">
         <v>52</v>
       </c>
@@ -1112,7 +1162,7 @@
       </c>
     </row>
     <row r="12" spans="1:4">
-      <c r="A12" s="34"/>
+      <c r="A12" s="32"/>
       <c r="B12" s="2" t="s">
         <v>4</v>
       </c>
@@ -1122,7 +1172,7 @@
       </c>
     </row>
     <row r="13" spans="1:4">
-      <c r="A13" s="34"/>
+      <c r="A13" s="32"/>
       <c r="B13" s="2" t="s">
         <v>5</v>
       </c>
@@ -1132,7 +1182,7 @@
       </c>
     </row>
     <row r="14" spans="1:4">
-      <c r="A14" s="34"/>
+      <c r="A14" s="32"/>
       <c r="B14" s="2" t="s">
         <v>6</v>
       </c>
@@ -1148,7 +1198,7 @@
       <c r="D15" s="25"/>
     </row>
     <row r="16" spans="1:4">
-      <c r="A16" s="34" t="s">
+      <c r="A16" s="32" t="s">
         <v>12</v>
       </c>
       <c r="B16" s="3" t="s">
@@ -1160,7 +1210,7 @@
       <c r="D16" s="4"/>
     </row>
     <row r="17" spans="1:4">
-      <c r="A17" s="34"/>
+      <c r="A17" s="32"/>
       <c r="B17" s="2" t="s">
         <v>8</v>
       </c>
@@ -1170,7 +1220,7 @@
       </c>
     </row>
     <row r="18" spans="1:4">
-      <c r="A18" s="34"/>
+      <c r="A18" s="32"/>
       <c r="B18" s="2" t="s">
         <v>9</v>
       </c>
@@ -1180,7 +1230,7 @@
       </c>
     </row>
     <row r="19" spans="1:4">
-      <c r="A19" s="34"/>
+      <c r="A19" s="32"/>
       <c r="B19" s="2" t="s">
         <v>62</v>
       </c>
@@ -1190,7 +1240,7 @@
       </c>
     </row>
     <row r="20" spans="1:4">
-      <c r="A20" s="34"/>
+      <c r="A20" s="32"/>
       <c r="B20" s="2" t="s">
         <v>64</v>
       </c>
@@ -1200,7 +1250,7 @@
       </c>
     </row>
     <row r="21" spans="1:4">
-      <c r="A21" s="34"/>
+      <c r="A21" s="32"/>
       <c r="B21" s="2" t="s">
         <v>67</v>
       </c>
@@ -1210,7 +1260,7 @@
       </c>
     </row>
     <row r="22" spans="1:4">
-      <c r="A22" s="34"/>
+      <c r="A22" s="32"/>
       <c r="B22" s="2" t="s">
         <v>70</v>
       </c>
@@ -1226,7 +1276,7 @@
       <c r="D23" s="1"/>
     </row>
     <row r="24" spans="1:4">
-      <c r="A24" s="34" t="s">
+      <c r="A24" s="32" t="s">
         <v>72</v>
       </c>
       <c r="B24" s="3" t="s">
@@ -1238,7 +1288,7 @@
       <c r="D24" s="27"/>
     </row>
     <row r="25" spans="1:4">
-      <c r="A25" s="34"/>
+      <c r="A25" s="32"/>
       <c r="B25" s="3" t="s">
         <v>75</v>
       </c>
@@ -1248,7 +1298,7 @@
       <c r="D25" s="27"/>
     </row>
     <row r="26" spans="1:4">
-      <c r="A26" s="34"/>
+      <c r="A26" s="32"/>
       <c r="B26" s="2" t="s">
         <v>76</v>
       </c>
@@ -1258,7 +1308,7 @@
       </c>
     </row>
     <row r="27" spans="1:4">
-      <c r="A27" s="34"/>
+      <c r="A27" s="32"/>
       <c r="B27" s="2" t="s">
         <v>78</v>
       </c>
@@ -1319,7 +1369,7 @@
       <c r="K1" s="13"/>
     </row>
     <row r="2" spans="1:11">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="34" t="s">
         <v>10</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1344,7 +1394,7 @@
       <c r="K2" s="14"/>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="37"/>
+      <c r="A3" s="35"/>
       <c r="B3" s="2" t="s">
         <v>34</v>
       </c>
@@ -1367,7 +1417,7 @@
       <c r="K3" s="14"/>
     </row>
     <row r="4" spans="1:11">
-      <c r="A4" s="37"/>
+      <c r="A4" s="35"/>
       <c r="B4" s="2" t="s">
         <v>38</v>
       </c>
@@ -1390,7 +1440,7 @@
       <c r="K4" s="14"/>
     </row>
     <row r="5" spans="1:11">
-      <c r="A5" s="38"/>
+      <c r="A5" s="36"/>
       <c r="B5" s="2" t="s">
         <v>40</v>
       </c>
@@ -1426,7 +1476,7 @@
       <c r="K6" s="14"/>
     </row>
     <row r="7" spans="1:11" ht="15" customHeight="1">
-      <c r="A7" s="39" t="s">
+      <c r="A7" s="37" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -1451,7 +1501,7 @@
       <c r="K7" s="14"/>
     </row>
     <row r="8" spans="1:11">
-      <c r="A8" s="40"/>
+      <c r="A8" s="38"/>
       <c r="B8" s="3" t="s">
         <v>46</v>
       </c>
@@ -1474,7 +1524,7 @@
       <c r="K8" s="14"/>
     </row>
     <row r="9" spans="1:11">
-      <c r="A9" s="40"/>
+      <c r="A9" s="38"/>
       <c r="B9" s="2" t="s">
         <v>48</v>
       </c>
@@ -1497,7 +1547,7 @@
       <c r="K9" s="14"/>
     </row>
     <row r="10" spans="1:11">
-      <c r="A10" s="40"/>
+      <c r="A10" s="38"/>
       <c r="B10" s="2" t="s">
         <v>50</v>
       </c>
@@ -1520,7 +1570,7 @@
       <c r="K10" s="14"/>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="40"/>
+      <c r="A11" s="38"/>
       <c r="B11" s="2" t="s">
         <v>52</v>
       </c>
@@ -1543,7 +1593,7 @@
       <c r="K11" s="14"/>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="40"/>
+      <c r="A12" s="38"/>
       <c r="B12" s="2" t="s">
         <v>4</v>
       </c>
@@ -1566,7 +1616,7 @@
       <c r="K12" s="14"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="40"/>
+      <c r="A13" s="38"/>
       <c r="B13" s="2" t="s">
         <v>5</v>
       </c>
@@ -1589,7 +1639,7 @@
       <c r="K13" s="14"/>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="41"/>
+      <c r="A14" s="39"/>
       <c r="B14" s="2" t="s">
         <v>6</v>
       </c>
@@ -1625,7 +1675,7 @@
       <c r="K15" s="14"/>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="39" t="s">
+      <c r="A16" s="37" t="s">
         <v>12</v>
       </c>
       <c r="B16" s="3" t="s">
@@ -1650,7 +1700,7 @@
       <c r="K16" s="14"/>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="40"/>
+      <c r="A17" s="38"/>
       <c r="B17" s="2" t="s">
         <v>8</v>
       </c>
@@ -1673,7 +1723,7 @@
       <c r="K17" s="14"/>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="40"/>
+      <c r="A18" s="38"/>
       <c r="B18" s="2" t="s">
         <v>9</v>
       </c>
@@ -1696,7 +1746,7 @@
       <c r="K18" s="14"/>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="40"/>
+      <c r="A19" s="38"/>
       <c r="B19" s="2" t="s">
         <v>62</v>
       </c>
@@ -1719,7 +1769,7 @@
       <c r="K19" s="14"/>
     </row>
     <row r="20" spans="1:11">
-      <c r="A20" s="40"/>
+      <c r="A20" s="38"/>
       <c r="B20" s="2" t="s">
         <v>64</v>
       </c>
@@ -1742,7 +1792,7 @@
       <c r="K20" s="14"/>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="40"/>
+      <c r="A21" s="38"/>
       <c r="B21" s="2" t="s">
         <v>67</v>
       </c>
@@ -1765,7 +1815,7 @@
       <c r="K21" s="14"/>
     </row>
     <row r="22" spans="1:11">
-      <c r="A22" s="41"/>
+      <c r="A22" s="39"/>
       <c r="B22" s="2" t="s">
         <v>70</v>
       </c>
@@ -1801,7 +1851,7 @@
       <c r="K23" s="14"/>
     </row>
     <row r="24" spans="1:11">
-      <c r="A24" s="34" t="s">
+      <c r="A24" s="32" t="s">
         <v>72</v>
       </c>
       <c r="B24" s="3" t="s">
@@ -1826,7 +1876,7 @@
       <c r="K24" s="14"/>
     </row>
     <row r="25" spans="1:11">
-      <c r="A25" s="34"/>
+      <c r="A25" s="32"/>
       <c r="B25" s="2" t="s">
         <v>75</v>
       </c>
@@ -1849,7 +1899,7 @@
       <c r="K25" s="14"/>
     </row>
     <row r="26" spans="1:11">
-      <c r="A26" s="34"/>
+      <c r="A26" s="32"/>
       <c r="B26" s="2" t="s">
         <v>76</v>
       </c>
@@ -2460,7 +2510,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="26" customWidth="1"/>
@@ -2471,7 +2521,7 @@
       <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="29" t="s">
         <v>25</v>
       </c>
       <c r="C1" s="5" t="s">
@@ -2572,22 +2622,82 @@
       <c r="B9" s="22" t="s">
         <v>118</v>
       </c>
-      <c r="C9" s="31"/>
-      <c r="D9" s="31" t="s">
+      <c r="C9" s="7"/>
+      <c r="D9" s="7" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:4">
-      <c r="A10" s="29"/>
-      <c r="B10" s="29"/>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
+      <c r="A10" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7">
+        <v>7</v>
+      </c>
     </row>
     <row r="11" spans="1:4">
-      <c r="A11" s="29"/>
-      <c r="B11" s="29"/>
-      <c r="C11" s="29"/>
-      <c r="D11" s="29"/>
+      <c r="A11" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B11" s="21" t="s">
+        <v>140</v>
+      </c>
+      <c r="C11" s="8">
+        <v>8</v>
+      </c>
+      <c r="D11" s="8"/>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>141</v>
+      </c>
+      <c r="C12" s="8">
+        <v>9</v>
+      </c>
+      <c r="D12" s="8"/>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" s="21" t="s">
+        <v>142</v>
+      </c>
+      <c r="C13" s="8">
+        <v>19</v>
+      </c>
+      <c r="D13" s="8"/>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="21" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="21" t="s">
+        <v>143</v>
+      </c>
+      <c r="C14" s="8">
+        <v>20</v>
+      </c>
+      <c r="D14" s="8"/>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7">
+        <v>21</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2596,456 +2706,683 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="5" max="5" width="25.5703125" customWidth="1"/>
     <col min="6" max="6" width="22.140625" customWidth="1"/>
+    <col min="7" max="7" width="21.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" s="5" t="s">
         <v>80</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="9" t="s">
         <v>123</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>11</v>
-      </c>
       <c r="F1" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="G1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="40" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:9">
       <c r="A2" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="30" t="s">
         <v>109</v>
       </c>
-      <c r="C2" s="32" t="s">
+      <c r="C2" s="30" t="s">
         <v>113</v>
       </c>
       <c r="D2" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="E2" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="F2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="G2" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="G2" s="8">
+      <c r="H2" s="8">
         <v>18</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="I2" s="41" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:9">
       <c r="A3" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="B3" s="32" t="s">
+      <c r="B3" s="30" t="s">
         <v>109</v>
       </c>
-      <c r="C3" s="32" t="s">
+      <c r="C3" s="30" t="s">
         <v>114</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>14</v>
+        <v>142</v>
       </c>
       <c r="E3" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F3" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="G3" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="G3" s="8">
+      <c r="H3" s="8">
         <v>18</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="I3" s="41" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:9">
       <c r="A4" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B4" s="33" t="s">
+      <c r="B4" s="31" t="s">
         <v>109</v>
       </c>
-      <c r="C4" s="33" t="s">
+      <c r="C4" s="31" t="s">
         <v>116</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>14</v>
+        <v>139</v>
       </c>
       <c r="E4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="G4" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G4" s="7">
+      <c r="H4" s="7">
         <v>18</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="I4" s="7" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:9">
       <c r="A5" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="B5" s="33" t="s">
+      <c r="B5" s="31" t="s">
         <v>109</v>
       </c>
-      <c r="C5" s="33" t="s">
+      <c r="C5" s="31" t="s">
         <v>118</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>14</v>
+        <v>143</v>
       </c>
       <c r="E5" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F5" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G5" s="7">
+      <c r="H5" s="7">
         <v>18</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="I5" s="7" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:9">
       <c r="A6" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="30" t="s">
         <v>110</v>
       </c>
-      <c r="C6" s="32" t="s">
+      <c r="C6" s="30" t="s">
         <v>113</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>14</v>
+        <v>141</v>
       </c>
       <c r="E6" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="F6" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="G6" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="G6" s="8">
+      <c r="H6" s="8">
         <v>19</v>
       </c>
-      <c r="H6" s="8" t="s">
+      <c r="I6" s="8" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:9">
+      <c r="A7" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="31" t="s">
         <v>110</v>
       </c>
-      <c r="C7" s="32" t="s">
+      <c r="C7" s="31" t="s">
         <v>114</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E7" s="8" t="s">
+      <c r="D7" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="G7" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G7" s="8">
+      <c r="H7" s="7">
         <v>19</v>
       </c>
-      <c r="H7" s="8" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
+      <c r="I7" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
       <c r="A8" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="B8" s="33" t="s">
+      <c r="B8" s="31" t="s">
         <v>110</v>
       </c>
-      <c r="C8" s="33" t="s">
+      <c r="C8" s="31" t="s">
         <v>116</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>14</v>
+        <v>143</v>
       </c>
       <c r="E8" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="G8" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G8" s="7">
+      <c r="H8" s="7">
         <v>19</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="I8" s="7" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:9">
       <c r="A9" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="B9" s="33" t="s">
+      <c r="B9" s="31" t="s">
         <v>110</v>
       </c>
-      <c r="C9" s="33" t="s">
+      <c r="C9" s="31" t="s">
         <v>118</v>
       </c>
       <c r="D9" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="E9" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="F9" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="F9" s="7" t="s">
+      <c r="G9" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G9" s="7">
+      <c r="H9" s="7">
         <v>19</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="I9" s="7" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:9">
       <c r="A10" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B10" s="33" t="s">
+      <c r="B10" s="31" t="s">
         <v>111</v>
       </c>
-      <c r="C10" s="33" t="s">
+      <c r="C10" s="31" t="s">
         <v>113</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>14</v>
+        <v>139</v>
       </c>
       <c r="E10" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="G10" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G10" s="7">
+      <c r="H10" s="7">
         <v>17</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="I10" s="7" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:9">
       <c r="A11" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B11" s="33" t="s">
+      <c r="B11" s="31" t="s">
         <v>111</v>
       </c>
-      <c r="C11" s="33" t="s">
+      <c r="C11" s="31" t="s">
         <v>114</v>
       </c>
       <c r="D11" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="E11" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="F11" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="G11" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G11" s="7">
+      <c r="H11" s="7">
         <v>17</v>
       </c>
-      <c r="H11" s="7" t="s">
+      <c r="I11" s="7" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:9">
       <c r="A12" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="B12" s="33" t="s">
+      <c r="B12" s="31" t="s">
         <v>111</v>
       </c>
-      <c r="C12" s="33" t="s">
+      <c r="C12" s="31" t="s">
         <v>116</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>14</v>
+        <v>142</v>
       </c>
       <c r="E12" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="F12" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="G12" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G12" s="7">
+      <c r="H12" s="7">
         <v>17</v>
       </c>
-      <c r="H12" s="7" t="s">
+      <c r="I12" s="7" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:9">
       <c r="A13" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="B13" s="33" t="s">
+      <c r="B13" s="31" t="s">
         <v>111</v>
       </c>
-      <c r="C13" s="33" t="s">
+      <c r="C13" s="31" t="s">
         <v>118</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>14</v>
+        <v>143</v>
       </c>
       <c r="E13" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="G13" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G13" s="7">
+      <c r="H13" s="7">
         <v>17</v>
       </c>
-      <c r="H13" s="7" t="s">
+      <c r="I13" s="7" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:9">
       <c r="A14" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="B14" s="33" t="s">
+      <c r="B14" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="C14" s="33" t="s">
+      <c r="C14" s="31" t="s">
         <v>113</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>14</v>
+        <v>143</v>
       </c>
       <c r="E14" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="G14" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G14" s="7">
+      <c r="H14" s="7">
         <v>0</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="I14" s="7" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:9">
       <c r="A15" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="B15" s="33" t="s">
+      <c r="B15" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="C15" s="33" t="s">
+      <c r="C15" s="31" t="s">
         <v>114</v>
       </c>
       <c r="D15" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="E15" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E15" s="7" t="s">
+      <c r="F15" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="G15" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G15" s="7">
+      <c r="H15" s="7">
         <v>0</v>
       </c>
-      <c r="H15" s="7" t="s">
+      <c r="I15" s="7" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:9">
       <c r="A16" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B16" s="33" t="s">
+      <c r="B16" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="C16" s="33" t="s">
+      <c r="C16" s="31" t="s">
         <v>116</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>14</v>
+        <v>141</v>
       </c>
       <c r="E16" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="F16" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="G16" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G16" s="7">
+      <c r="H16" s="7">
         <v>0</v>
       </c>
-      <c r="H16" s="7" t="s">
+      <c r="I16" s="7" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:9">
       <c r="A17" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B17" s="33" t="s">
+      <c r="B17" s="31" t="s">
         <v>112</v>
       </c>
-      <c r="C17" s="33" t="s">
+      <c r="C17" s="31" t="s">
         <v>118</v>
       </c>
       <c r="D17" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="H17" s="7">
+        <v>0</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="B18" s="42" t="s">
+        <v>109</v>
+      </c>
+      <c r="C18" s="42" t="s">
+        <v>113</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>142</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>154</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="H18" s="8">
+        <v>18</v>
+      </c>
+      <c r="I18" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="B19" s="42" t="s">
+        <v>110</v>
+      </c>
+      <c r="C19" s="42" t="s">
+        <v>114</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="E19" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E17" s="7" t="s">
+      <c r="F19" s="8" t="s">
+        <v>115</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="H19" s="8">
+        <v>19</v>
+      </c>
+      <c r="I19" s="8" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="B20" s="43" t="s">
+        <v>111</v>
+      </c>
+      <c r="C20" s="43" t="s">
+        <v>116</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="H20" s="7">
+        <v>17</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="B21" s="43" t="s">
+        <v>112</v>
+      </c>
+      <c r="C21" s="43" t="s">
+        <v>118</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="G21" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="G17" s="7">
+      <c r="H21" s="7">
         <v>0</v>
       </c>
-      <c r="H17" s="7" t="s">
+      <c r="I21" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="B22" s="43" t="s">
+        <v>109</v>
+      </c>
+      <c r="C22" s="43" t="s">
+        <v>116</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="H22" s="7">
+        <v>18</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="B23" s="43" t="s">
+        <v>110</v>
+      </c>
+      <c r="C23" s="43" t="s">
+        <v>118</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>154</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="H23" s="7">
+        <v>19</v>
+      </c>
+      <c r="I23" s="7" t="s">
         <v>107</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>